<commit_message>
ran implied and mercec weights
</commit_message>
<xml_diff>
--- a/Scoring Logic and Documentation/method/implied_weights_summary.xlsx
+++ b/Scoring Logic and Documentation/method/implied_weights_summary.xlsx
@@ -473,19 +473,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.212229</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0.3</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.087771</v>
+        <v>-0.3</v>
       </c>
       <c r="G2" t="n">
-        <v>0.952</v>
+        <v>0.752</v>
       </c>
       <c r="H2" t="n">
-        <v>0.603</v>
+        <v>0.0259</v>
       </c>
     </row>
     <row r="3">
@@ -503,19 +503,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.418194</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0.35</v>
       </c>
       <c r="F3" t="n">
-        <v>0.068194</v>
+        <v>-0.35</v>
       </c>
       <c r="G3" t="n">
-        <v>0.952</v>
+        <v>0.752</v>
       </c>
       <c r="H3" t="n">
-        <v>0.603</v>
+        <v>0.0259</v>
       </c>
     </row>
     <row r="4">
@@ -533,19 +533,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.292554</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>0.2</v>
       </c>
       <c r="F4" t="n">
-        <v>0.092554</v>
+        <v>0.8</v>
       </c>
       <c r="G4" t="n">
-        <v>0.952</v>
+        <v>0.752</v>
       </c>
       <c r="H4" t="n">
-        <v>0.603</v>
+        <v>0.0259</v>
       </c>
     </row>
     <row r="5">
@@ -563,19 +563,19 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.07702299999999999</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0.15</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.072977</v>
+        <v>-0.15</v>
       </c>
       <c r="G5" t="n">
-        <v>0.952</v>
+        <v>0.752</v>
       </c>
       <c r="H5" t="n">
-        <v>0.603</v>
+        <v>0.0259</v>
       </c>
     </row>
     <row r="6">
@@ -593,19 +593,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.621198</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>0.3</v>
       </c>
       <c r="F6" t="n">
-        <v>0.321198</v>
+        <v>-0.3</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9333</v>
+        <v>0.854</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7159</v>
+        <v>0.285</v>
       </c>
     </row>
     <row r="7">
@@ -632,10 +632,10 @@
         <v>-0.35</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9333</v>
+        <v>0.854</v>
       </c>
       <c r="H7" t="n">
-        <v>0.7159</v>
+        <v>0.285</v>
       </c>
     </row>
     <row r="8">
@@ -653,19 +653,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.378802</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>0.2</v>
       </c>
       <c r="F8" t="n">
-        <v>0.178802</v>
+        <v>0.8</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9333</v>
+        <v>0.854</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7159</v>
+        <v>0.285</v>
       </c>
     </row>
     <row r="9">
@@ -692,10 +692,10 @@
         <v>-0.15</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9333</v>
+        <v>0.854</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7159</v>
+        <v>0.285</v>
       </c>
     </row>
     <row r="10">
@@ -713,19 +713,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.183821</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
         <v>0.3</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.116179</v>
+        <v>-0.3</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9633</v>
+        <v>0.92</v>
       </c>
       <c r="H10" t="n">
-        <v>0.5891999999999999</v>
+        <v>-0.2108</v>
       </c>
     </row>
     <row r="11">
@@ -743,19 +743,19 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.507355</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0.35</v>
       </c>
       <c r="F11" t="n">
-        <v>0.157355</v>
+        <v>-0.35</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9633</v>
+        <v>0.92</v>
       </c>
       <c r="H11" t="n">
-        <v>0.5891999999999999</v>
+        <v>-0.2108</v>
       </c>
     </row>
     <row r="12">
@@ -773,19 +773,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.117213</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0.2</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.082787</v>
+        <v>-0.2</v>
       </c>
       <c r="G12" t="n">
-        <v>0.9633</v>
+        <v>0.92</v>
       </c>
       <c r="H12" t="n">
-        <v>0.5891999999999999</v>
+        <v>-0.2108</v>
       </c>
     </row>
     <row r="13">
@@ -803,19 +803,19 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.191611</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
         <v>0.15</v>
       </c>
       <c r="F13" t="n">
-        <v>0.041611</v>
+        <v>0.85</v>
       </c>
       <c r="G13" t="n">
-        <v>0.9633</v>
+        <v>0.92</v>
       </c>
       <c r="H13" t="n">
-        <v>0.5891999999999999</v>
+        <v>-0.2108</v>
       </c>
     </row>
     <row r="14">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.253025</v>
+        <v>0.211194</v>
       </c>
       <c r="E14" t="n">
         <v>0.3</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.046975</v>
+        <v>-0.088806</v>
       </c>
       <c r="G14" t="n">
-        <v>0.9208</v>
+        <v>0.8375</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4904</v>
+        <v>-0.2868</v>
       </c>
     </row>
     <row r="15">
@@ -863,19 +863,19 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.4002</v>
+        <v>0.788806</v>
       </c>
       <c r="E15" t="n">
         <v>0.35</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0502</v>
+        <v>0.438806</v>
       </c>
       <c r="G15" t="n">
-        <v>0.9208</v>
+        <v>0.8375</v>
       </c>
       <c r="H15" t="n">
-        <v>0.4904</v>
+        <v>-0.2868</v>
       </c>
     </row>
     <row r="16">
@@ -893,19 +893,19 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.049761</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
         <v>0.2</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.150239</v>
+        <v>-0.2</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9208</v>
+        <v>0.8375</v>
       </c>
       <c r="H16" t="n">
-        <v>0.4904</v>
+        <v>-0.2868</v>
       </c>
     </row>
     <row r="17">
@@ -923,19 +923,19 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.297014</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
         <v>0.15</v>
       </c>
       <c r="F17" t="n">
-        <v>0.147014</v>
+        <v>-0.15</v>
       </c>
       <c r="G17" t="n">
-        <v>0.9208</v>
+        <v>0.8375</v>
       </c>
       <c r="H17" t="n">
-        <v>0.4904</v>
+        <v>-0.2868</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ran remaining weight analysis scripts, then udpated RunRagAbalations to rely on the represetnative sampling.
</commit_message>
<xml_diff>
--- a/Scoring Logic and Documentation/method/implied_weights_summary.xlsx
+++ b/Scoring Logic and Documentation/method/implied_weights_summary.xlsx
@@ -722,7 +722,7 @@
         <v>-0.3</v>
       </c>
       <c r="G10" t="n">
-        <v>0.92</v>
+        <v>0.9167</v>
       </c>
       <c r="H10" t="n">
         <v>-0.2108</v>
@@ -752,7 +752,7 @@
         <v>-0.35</v>
       </c>
       <c r="G11" t="n">
-        <v>0.92</v>
+        <v>0.9167</v>
       </c>
       <c r="H11" t="n">
         <v>-0.2108</v>
@@ -782,7 +782,7 @@
         <v>-0.2</v>
       </c>
       <c r="G12" t="n">
-        <v>0.92</v>
+        <v>0.9167</v>
       </c>
       <c r="H12" t="n">
         <v>-0.2108</v>
@@ -812,7 +812,7 @@
         <v>0.85</v>
       </c>
       <c r="G13" t="n">
-        <v>0.92</v>
+        <v>0.9167</v>
       </c>
       <c r="H13" t="n">
         <v>-0.2108</v>

</xml_diff>